<commit_message>
Add Design section (P4): sequence diagrams, API design, error handling, UX
- SAD v1.2: Section 4 filled (SD-01 Login, SD-02 Attempt Exam, SD-03 Submit Exam,
  API catalogue + 4 detailed endpoints, error/logging/monitoring, UX, design traceability)
- Design/diagrams: Mermaid sources + rendered PNGs
- RTM: filled 'Design / API ref - P4' column for all 53 requirements
</commit_message>
<xml_diff>
--- a/SRS/RTM_Online_Exam_Portal.xlsx
+++ b/SRS/RTM_Online_Exam_Portal.xlsx
@@ -582,7 +582,11 @@
       <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="3" t="inlineStr"/>
       <c r="I2" s="3" t="inlineStr"/>
-      <c r="J2" s="3" t="inlineStr"/>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>§4.3 API-01; services/auth</t>
+        </is>
+      </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -623,7 +627,11 @@
       <c r="G3" s="4" t="inlineStr"/>
       <c r="H3" s="3" t="inlineStr"/>
       <c r="I3" s="3" t="inlineStr"/>
-      <c r="J3" s="3" t="inlineStr"/>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>§4.3 API-02; services/auth + notification</t>
+        </is>
+      </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -664,7 +672,11 @@
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="3" t="inlineStr"/>
       <c r="I4" s="3" t="inlineStr"/>
-      <c r="J4" s="3" t="inlineStr"/>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>§4.2 SD-01; §4.3 API-03</t>
+        </is>
+      </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -705,7 +717,11 @@
       <c r="G5" s="4" t="inlineStr"/>
       <c r="H5" s="3" t="inlineStr"/>
       <c r="I5" s="3" t="inlineStr"/>
-      <c r="J5" s="3" t="inlineStr"/>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>§4.2 SD-01; §4.3 API-04</t>
+        </is>
+      </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -746,7 +762,11 @@
       <c r="G6" s="2" t="inlineStr"/>
       <c r="H6" s="3" t="inlineStr"/>
       <c r="I6" s="3" t="inlineStr"/>
-      <c r="J6" s="3" t="inlineStr"/>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>§4.3 API-05, API-06</t>
+        </is>
+      </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -787,7 +807,11 @@
       <c r="G7" s="4" t="inlineStr"/>
       <c r="H7" s="3" t="inlineStr"/>
       <c r="I7" s="3" t="inlineStr"/>
-      <c r="J7" s="3" t="inlineStr"/>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>§4.3 API-07</t>
+        </is>
+      </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -828,7 +852,11 @@
       <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="3" t="inlineStr"/>
       <c r="I8" s="3" t="inlineStr"/>
-      <c r="J8" s="3" t="inlineStr"/>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>§4.3 API-08; §4.1 questions collection</t>
+        </is>
+      </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -869,7 +897,11 @@
       <c r="G9" s="4" t="inlineStr"/>
       <c r="H9" s="3" t="inlineStr"/>
       <c r="I9" s="3" t="inlineStr"/>
-      <c r="J9" s="3" t="inlineStr"/>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>§4.3 API-09; §4.1 exams collection</t>
+        </is>
+      </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -910,7 +942,11 @@
       <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="3" t="inlineStr"/>
       <c r="I10" s="3" t="inlineStr"/>
-      <c r="J10" s="3" t="inlineStr"/>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>§4.3 API-09; §4.2 SD-02 (shuffle)</t>
+        </is>
+      </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -951,7 +987,11 @@
       <c r="G11" s="4" t="inlineStr"/>
       <c r="H11" s="3" t="inlineStr"/>
       <c r="I11" s="3" t="inlineStr"/>
-      <c r="J11" s="3" t="inlineStr"/>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>§4.3 API-09; §4.2 SD-03 (negative marking)</t>
+        </is>
+      </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -992,7 +1032,11 @@
       <c r="G12" s="2" t="inlineStr"/>
       <c r="H12" s="3" t="inlineStr"/>
       <c r="I12" s="3" t="inlineStr"/>
-      <c r="J12" s="3" t="inlineStr"/>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>§4.3 API-10</t>
+        </is>
+      </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -1033,7 +1077,11 @@
       <c r="G13" s="4" t="inlineStr"/>
       <c r="H13" s="3" t="inlineStr"/>
       <c r="I13" s="3" t="inlineStr"/>
-      <c r="J13" s="3" t="inlineStr"/>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>§4.2 SD-02 (exam.locked); §4.3 API-09 (409 EXAM_LOCKED)</t>
+        </is>
+      </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -1074,7 +1122,11 @@
       <c r="G14" s="2" t="inlineStr"/>
       <c r="H14" s="3" t="inlineStr"/>
       <c r="I14" s="3" t="inlineStr"/>
-      <c r="J14" s="3" t="inlineStr"/>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>§4.3 API-11; §4.5 Student dashboard</t>
+        </is>
+      </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -1115,7 +1167,11 @@
       <c r="G15" s="4" t="inlineStr"/>
       <c r="H15" s="3" t="inlineStr"/>
       <c r="I15" s="3" t="inlineStr"/>
-      <c r="J15" s="3" t="inlineStr"/>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>§4.2 SD-02; §4.3 API-12</t>
+        </is>
+      </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -1156,7 +1212,11 @@
       <c r="G16" s="2" t="inlineStr"/>
       <c r="H16" s="3" t="inlineStr"/>
       <c r="I16" s="3" t="inlineStr"/>
-      <c r="J16" s="3" t="inlineStr"/>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>§4.2 SD-02; §4.3 API-13; §4.5 Question panel</t>
+        </is>
+      </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -1197,7 +1257,11 @@
       <c r="G17" s="4" t="inlineStr"/>
       <c r="H17" s="3" t="inlineStr"/>
       <c r="I17" s="3" t="inlineStr"/>
-      <c r="J17" s="3" t="inlineStr"/>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>§4.2 SD-02; §4.3 API-12 (endsAt/serverTime); §4.5 Timer</t>
+        </is>
+      </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -1238,7 +1302,11 @@
       <c r="G18" s="2" t="inlineStr"/>
       <c r="H18" s="3" t="inlineStr"/>
       <c r="I18" s="3" t="inlineStr"/>
-      <c r="J18" s="3" t="inlineStr"/>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>§4.2 SD-02; §4.3 API-13</t>
+        </is>
+      </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -1279,7 +1347,11 @@
       <c r="G19" s="4" t="inlineStr"/>
       <c r="H19" s="3" t="inlineStr"/>
       <c r="I19" s="3" t="inlineStr"/>
-      <c r="J19" s="3" t="inlineStr"/>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>§4.2 SD-02 (resume); §4.3 API-12</t>
+        </is>
+      </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -1320,7 +1392,11 @@
       <c r="G20" s="2" t="inlineStr"/>
       <c r="H20" s="3" t="inlineStr"/>
       <c r="I20" s="3" t="inlineStr"/>
-      <c r="J20" s="3" t="inlineStr"/>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>§4.2 SD-03; §4.3 API-15; §4.5 Submit dialog</t>
+        </is>
+      </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -1361,7 +1437,11 @@
       <c r="G21" s="4" t="inlineStr"/>
       <c r="H21" s="3" t="inlineStr"/>
       <c r="I21" s="3" t="inlineStr"/>
-      <c r="J21" s="3" t="inlineStr"/>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>§4.2 SD-03 (auto-submit job); §4.3 API-15; M-06</t>
+        </is>
+      </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -1402,7 +1482,11 @@
       <c r="G22" s="2" t="inlineStr"/>
       <c r="H22" s="3" t="inlineStr"/>
       <c r="I22" s="3" t="inlineStr"/>
-      <c r="J22" s="3" t="inlineStr"/>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>§4.2 SD-02; §4.3 API-14, API-17</t>
+        </is>
+      </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -1443,7 +1527,11 @@
       <c r="G23" s="4" t="inlineStr"/>
       <c r="H23" s="3" t="inlineStr"/>
       <c r="I23" s="3" t="inlineStr"/>
-      <c r="J23" s="3" t="inlineStr"/>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>§4.2 SD-03; §4.3 API-15</t>
+        </is>
+      </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -1484,7 +1572,11 @@
       <c r="G24" s="2" t="inlineStr"/>
       <c r="H24" s="3" t="inlineStr"/>
       <c r="I24" s="3" t="inlineStr"/>
-      <c r="J24" s="3" t="inlineStr"/>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>§4.3 API-16; §4.5 Result page</t>
+        </is>
+      </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -1525,7 +1617,11 @@
       <c r="G25" s="4" t="inlineStr"/>
       <c r="H25" s="3" t="inlineStr"/>
       <c r="I25" s="3" t="inlineStr"/>
-      <c r="J25" s="3" t="inlineStr"/>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>§4.3 API-17</t>
+        </is>
+      </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -1566,7 +1662,11 @@
       <c r="G26" s="2" t="inlineStr"/>
       <c r="H26" s="3" t="inlineStr"/>
       <c r="I26" s="3" t="inlineStr"/>
-      <c r="J26" s="3" t="inlineStr"/>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>§4.3 API-18</t>
+        </is>
+      </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -1607,7 +1707,11 @@
       <c r="G27" s="4" t="inlineStr"/>
       <c r="H27" s="3" t="inlineStr"/>
       <c r="I27" s="3" t="inlineStr"/>
-      <c r="J27" s="3" t="inlineStr"/>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>§4.2 SD-03; §4.3 API-10, API-19</t>
+        </is>
+      </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -1648,7 +1752,11 @@
       <c r="G28" s="2" t="inlineStr"/>
       <c r="H28" s="3" t="inlineStr"/>
       <c r="I28" s="3" t="inlineStr"/>
-      <c r="J28" s="3" t="inlineStr"/>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>§4.3 API-20; §4.4.2 Audit log</t>
+        </is>
+      </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -1685,7 +1793,11 @@
       <c r="G29" s="4" t="inlineStr"/>
       <c r="H29" s="3" t="inlineStr"/>
       <c r="I29" s="3" t="inlineStr"/>
-      <c r="J29" s="3" t="inlineStr"/>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>§4.4.3 M-01</t>
+        </is>
+      </c>
       <c r="K29" s="4" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -1722,7 +1834,11 @@
       <c r="G30" s="2" t="inlineStr"/>
       <c r="H30" s="3" t="inlineStr"/>
       <c r="I30" s="3" t="inlineStr"/>
-      <c r="J30" s="3" t="inlineStr"/>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>§4.3 API-13; §4.4.3 M-02</t>
+        </is>
+      </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -1759,7 +1875,11 @@
       <c r="G31" s="4" t="inlineStr"/>
       <c r="H31" s="3" t="inlineStr"/>
       <c r="I31" s="3" t="inlineStr"/>
-      <c r="J31" s="3" t="inlineStr"/>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>§4.2 SD-03; §4.4.3 M-03</t>
+        </is>
+      </c>
       <c r="K31" s="4" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -1796,7 +1916,11 @@
       <c r="G32" s="2" t="inlineStr"/>
       <c r="H32" s="3" t="inlineStr"/>
       <c r="I32" s="3" t="inlineStr"/>
-      <c r="J32" s="3" t="inlineStr"/>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>§4.3 API-21; §4.4.3 M-04, M-05</t>
+        </is>
+      </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -1833,7 +1957,11 @@
       <c r="G33" s="4" t="inlineStr"/>
       <c r="H33" s="3" t="inlineStr"/>
       <c r="I33" s="3" t="inlineStr"/>
-      <c r="J33" s="3" t="inlineStr"/>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>§4.2 SD-02, SD-03; §4.4.1 exam-page resilience</t>
+        </is>
+      </c>
       <c r="K33" s="4" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -1870,7 +1998,11 @@
       <c r="G34" s="2" t="inlineStr"/>
       <c r="H34" s="3" t="inlineStr"/>
       <c r="I34" s="3" t="inlineStr"/>
-      <c r="J34" s="3" t="inlineStr"/>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>§4.1 jobs/backup; §4.4.3 M-08</t>
+        </is>
+      </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -1907,7 +2039,11 @@
       <c r="G35" s="4" t="inlineStr"/>
       <c r="H35" s="3" t="inlineStr"/>
       <c r="I35" s="3" t="inlineStr"/>
-      <c r="J35" s="3" t="inlineStr"/>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>§4.5 Student dashboard (3 clicks)</t>
+        </is>
+      </c>
       <c r="K35" s="4" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -1944,7 +2080,11 @@
       <c r="G36" s="2" t="inlineStr"/>
       <c r="H36" s="3" t="inlineStr"/>
       <c r="I36" s="3" t="inlineStr"/>
-      <c r="J36" s="3" t="inlineStr"/>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>§4.5 Accessibility</t>
+        </is>
+      </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -1981,7 +2121,11 @@
       <c r="G37" s="4" t="inlineStr"/>
       <c r="H37" s="3" t="inlineStr"/>
       <c r="I37" s="3" t="inlineStr"/>
-      <c r="J37" s="3" t="inlineStr"/>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>§4.5 Accessibility &amp; compatibility</t>
+        </is>
+      </c>
       <c r="K37" s="4" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -2018,7 +2162,11 @@
       <c r="G38" s="2" t="inlineStr"/>
       <c r="H38" s="3" t="inlineStr"/>
       <c r="I38" s="3" t="inlineStr"/>
-      <c r="J38" s="3" t="inlineStr"/>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>§4.2 SD-02 (server time offset); §4.3 API-12</t>
+        </is>
+      </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -2055,7 +2203,11 @@
       <c r="G39" s="4" t="inlineStr"/>
       <c r="H39" s="3" t="inlineStr"/>
       <c r="I39" s="3" t="inlineStr"/>
-      <c r="J39" s="3" t="inlineStr"/>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>§4.1 data entities &amp; indexes</t>
+        </is>
+      </c>
       <c r="K39" s="4" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -2092,7 +2244,11 @@
       <c r="G40" s="2" t="inlineStr"/>
       <c r="H40" s="3" t="inlineStr"/>
       <c r="I40" s="3" t="inlineStr"/>
-      <c r="J40" s="3" t="inlineStr"/>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>§4.1 module structure</t>
+        </is>
+      </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -2129,7 +2285,11 @@
       <c r="G41" s="4" t="inlineStr"/>
       <c r="H41" s="3" t="inlineStr"/>
       <c r="I41" s="3" t="inlineStr"/>
-      <c r="J41" s="3" t="inlineStr"/>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>§4.7 item 5 (Docker Compose)</t>
+        </is>
+      </c>
       <c r="K41" s="4" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -2166,7 +2326,11 @@
       <c r="G42" s="2" t="inlineStr"/>
       <c r="H42" s="3" t="inlineStr"/>
       <c r="I42" s="3" t="inlineStr"/>
-      <c r="J42" s="3" t="inlineStr"/>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>§4.3 API-07; §4.1 data entities</t>
+        </is>
+      </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -2207,7 +2371,11 @@
       </c>
       <c r="H43" s="3" t="inlineStr"/>
       <c r="I43" s="3" t="inlineStr"/>
-      <c r="J43" s="3" t="inlineStr"/>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>§4.2 SD-01; §4.3 API-03</t>
+        </is>
+      </c>
       <c r="K43" s="4" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -2248,7 +2416,11 @@
       </c>
       <c r="H44" s="3" t="inlineStr"/>
       <c r="I44" s="3" t="inlineStr"/>
-      <c r="J44" s="3" t="inlineStr"/>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>§4.3 API-01, API-06</t>
+        </is>
+      </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -2289,7 +2461,11 @@
       </c>
       <c r="H45" s="3" t="inlineStr"/>
       <c r="I45" s="3" t="inlineStr"/>
-      <c r="J45" s="3" t="inlineStr"/>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>§4.2 SD-01; §4.3 API-03 (423)</t>
+        </is>
+      </c>
       <c r="K45" s="4" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -2330,7 +2506,11 @@
       </c>
       <c r="H46" s="3" t="inlineStr"/>
       <c r="I46" s="3" t="inlineStr"/>
-      <c r="J46" s="3" t="inlineStr"/>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>§4.2 SD-01, SD-02; §4.3.1 conventions</t>
+        </is>
+      </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -2371,7 +2551,11 @@
       </c>
       <c r="H47" s="3" t="inlineStr"/>
       <c r="I47" s="3" t="inlineStr"/>
-      <c r="J47" s="3" t="inlineStr"/>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>§4.3.1 conventions</t>
+        </is>
+      </c>
       <c r="K47" s="4" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -2412,7 +2596,11 @@
       </c>
       <c r="H48" s="3" t="inlineStr"/>
       <c r="I48" s="3" t="inlineStr"/>
-      <c r="J48" s="3" t="inlineStr"/>
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>§4.2 SD-01; §4.3 API-03</t>
+        </is>
+      </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -2453,7 +2641,11 @@
       </c>
       <c r="H49" s="3" t="inlineStr"/>
       <c r="I49" s="3" t="inlineStr"/>
-      <c r="J49" s="3" t="inlineStr"/>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>§4.2 SD-02; §4.3 API-12, API-16</t>
+        </is>
+      </c>
       <c r="K49" s="4" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -2494,7 +2686,11 @@
       </c>
       <c r="H50" s="3" t="inlineStr"/>
       <c r="I50" s="3" t="inlineStr"/>
-      <c r="J50" s="3" t="inlineStr"/>
+      <c r="J50" s="3" t="inlineStr">
+        <is>
+          <t>§4.3.1 conventions; §4.4.1</t>
+        </is>
+      </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -2535,7 +2731,11 @@
       </c>
       <c r="H51" s="3" t="inlineStr"/>
       <c r="I51" s="3" t="inlineStr"/>
-      <c r="J51" s="3" t="inlineStr"/>
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>§4.2 SD-02, SD-03; §4.3 API-13, API-15</t>
+        </is>
+      </c>
       <c r="K51" s="4" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -2576,7 +2776,11 @@
       </c>
       <c r="H52" s="3" t="inlineStr"/>
       <c r="I52" s="3" t="inlineStr"/>
-      <c r="J52" s="3" t="inlineStr"/>
+      <c r="J52" s="3" t="inlineStr">
+        <is>
+          <t>§4.2 SD-01; §4.3 API-03, API-05 (429)</t>
+        </is>
+      </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -2617,7 +2821,11 @@
       </c>
       <c r="H53" s="3" t="inlineStr"/>
       <c r="I53" s="3" t="inlineStr"/>
-      <c r="J53" s="3" t="inlineStr"/>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>§4.4.2 Logging; §4.3 API-20</t>
+        </is>
+      </c>
       <c r="K53" s="4" t="inlineStr">
         <is>
           <t>Drafted</t>
@@ -2658,7 +2866,11 @@
       </c>
       <c r="H54" s="3" t="inlineStr"/>
       <c r="I54" s="3" t="inlineStr"/>
-      <c r="J54" s="3" t="inlineStr"/>
+      <c r="J54" s="3" t="inlineStr">
+        <is>
+          <t>§4.1 data entities (encrypted fields)</t>
+        </is>
+      </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
           <t>Drafted</t>

</xml_diff>

<commit_message>
RTM: add architecture components (P3)
</commit_message>
<xml_diff>
--- a/SRS/RTM_Online_Exam_Portal.xlsx
+++ b/SRS/RTM_Online_Exam_Portal.xlsx
@@ -581,7 +581,11 @@
       </c>
       <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="3" t="inlineStr"/>
-      <c r="I2" s="3" t="inlineStr"/>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Authentication &amp; Authorization Service</t>
+        </is>
+      </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
           <t>§4.3 API-01; services/auth</t>
@@ -626,7 +630,11 @@
       </c>
       <c r="G3" s="4" t="inlineStr"/>
       <c r="H3" s="3" t="inlineStr"/>
-      <c r="I3" s="3" t="inlineStr"/>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Authentication &amp; Authorization Service + Notification Service</t>
+        </is>
+      </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
           <t>§4.3 API-02; services/auth + notification</t>
@@ -671,7 +679,11 @@
       </c>
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Authentication &amp; Authorization Service</t>
+        </is>
+      </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
           <t>§4.2 SD-01; §4.3 API-03</t>
@@ -716,7 +728,11 @@
       </c>
       <c r="G5" s="4" t="inlineStr"/>
       <c r="H5" s="3" t="inlineStr"/>
-      <c r="I5" s="3" t="inlineStr"/>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Authentication &amp; Authorization Service</t>
+        </is>
+      </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
           <t>§4.2 SD-01; §4.3 API-04</t>
@@ -761,7 +777,11 @@
       </c>
       <c r="G6" s="2" t="inlineStr"/>
       <c r="H6" s="3" t="inlineStr"/>
-      <c r="I6" s="3" t="inlineStr"/>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>Authentication &amp; Authorization Service + Notification Service</t>
+        </is>
+      </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
           <t>§4.3 API-05, API-06</t>
@@ -806,7 +826,11 @@
       </c>
       <c r="G7" s="4" t="inlineStr"/>
       <c r="H7" s="3" t="inlineStr"/>
-      <c r="I7" s="3" t="inlineStr"/>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Authentication &amp; Authorization Service</t>
+        </is>
+      </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
           <t>§4.3 API-07</t>
@@ -851,7 +875,11 @@
       </c>
       <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="3" t="inlineStr"/>
-      <c r="I8" s="3" t="inlineStr"/>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>Question Bank Service</t>
+        </is>
+      </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
           <t>§4.3 API-08; §4.1 questions collection</t>
@@ -896,7 +924,11 @@
       </c>
       <c r="G9" s="4" t="inlineStr"/>
       <c r="H9" s="3" t="inlineStr"/>
-      <c r="I9" s="3" t="inlineStr"/>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Exam Management Service</t>
+        </is>
+      </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
           <t>§4.3 API-09; §4.1 exams collection</t>
@@ -941,7 +973,11 @@
       </c>
       <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="3" t="inlineStr"/>
-      <c r="I10" s="3" t="inlineStr"/>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Exam Management Service</t>
+        </is>
+      </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
           <t>§4.3 API-09; §4.2 SD-02 (shuffle)</t>
@@ -986,7 +1022,11 @@
       </c>
       <c r="G11" s="4" t="inlineStr"/>
       <c r="H11" s="3" t="inlineStr"/>
-      <c r="I11" s="3" t="inlineStr"/>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Exam Management Service + Evaluation Engine</t>
+        </is>
+      </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
           <t>§4.3 API-09; §4.2 SD-03 (negative marking)</t>
@@ -1031,7 +1071,11 @@
       </c>
       <c r="G12" s="2" t="inlineStr"/>
       <c r="H12" s="3" t="inlineStr"/>
-      <c r="I12" s="3" t="inlineStr"/>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>Exam Management Service + Notification Service</t>
+        </is>
+      </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
           <t>§4.3 API-10</t>
@@ -1076,7 +1120,11 @@
       </c>
       <c r="G13" s="4" t="inlineStr"/>
       <c r="H13" s="3" t="inlineStr"/>
-      <c r="I13" s="3" t="inlineStr"/>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Exam Management Service</t>
+        </is>
+      </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
           <t>§4.2 SD-02 (exam.locked); §4.3 API-09 (409 EXAM_LOCKED)</t>
@@ -1121,7 +1169,11 @@
       </c>
       <c r="G14" s="2" t="inlineStr"/>
       <c r="H14" s="3" t="inlineStr"/>
-      <c r="I14" s="3" t="inlineStr"/>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>Exam Management Service</t>
+        </is>
+      </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
           <t>§4.3 API-11; §4.5 Student dashboard</t>
@@ -1166,7 +1218,11 @@
       </c>
       <c r="G15" s="4" t="inlineStr"/>
       <c r="H15" s="3" t="inlineStr"/>
-      <c r="I15" s="3" t="inlineStr"/>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Exam Management Service</t>
+        </is>
+      </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
           <t>§4.2 SD-02; §4.3 API-12</t>
@@ -1211,7 +1267,11 @@
       </c>
       <c r="G16" s="2" t="inlineStr"/>
       <c r="H16" s="3" t="inlineStr"/>
-      <c r="I16" s="3" t="inlineStr"/>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>Exam Management Service + Presentation Layer</t>
+        </is>
+      </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
           <t>§4.2 SD-02; §4.3 API-13; §4.5 Question panel</t>
@@ -1256,7 +1316,11 @@
       </c>
       <c r="G17" s="4" t="inlineStr"/>
       <c r="H17" s="3" t="inlineStr"/>
-      <c r="I17" s="3" t="inlineStr"/>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Exam Management Service</t>
+        </is>
+      </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
           <t>§4.2 SD-02; §4.3 API-12 (endsAt/serverTime); §4.5 Timer</t>
@@ -1301,7 +1365,11 @@
       </c>
       <c r="G18" s="2" t="inlineStr"/>
       <c r="H18" s="3" t="inlineStr"/>
-      <c r="I18" s="3" t="inlineStr"/>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>Exam Management Service</t>
+        </is>
+      </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
           <t>§4.2 SD-02; §4.3 API-13</t>
@@ -1346,7 +1414,11 @@
       </c>
       <c r="G19" s="4" t="inlineStr"/>
       <c r="H19" s="3" t="inlineStr"/>
-      <c r="I19" s="3" t="inlineStr"/>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Exam Management Service</t>
+        </is>
+      </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
           <t>§4.2 SD-02 (resume); §4.3 API-12</t>
@@ -1391,7 +1463,11 @@
       </c>
       <c r="G20" s="2" t="inlineStr"/>
       <c r="H20" s="3" t="inlineStr"/>
-      <c r="I20" s="3" t="inlineStr"/>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>Exam Management Service</t>
+        </is>
+      </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
           <t>§4.2 SD-03; §4.3 API-15; §4.5 Submit dialog</t>
@@ -1436,7 +1512,11 @@
       </c>
       <c r="G21" s="4" t="inlineStr"/>
       <c r="H21" s="3" t="inlineStr"/>
-      <c r="I21" s="3" t="inlineStr"/>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Exam Management Service</t>
+        </is>
+      </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
           <t>§4.2 SD-03 (auto-submit job); §4.3 API-15; M-06</t>
@@ -1481,7 +1561,11 @@
       </c>
       <c r="G22" s="2" t="inlineStr"/>
       <c r="H22" s="3" t="inlineStr"/>
-      <c r="I22" s="3" t="inlineStr"/>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>Exam Management Service + Audit &amp; Logging Service</t>
+        </is>
+      </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
           <t>§4.2 SD-02; §4.3 API-14, API-17</t>
@@ -1526,7 +1610,11 @@
       </c>
       <c r="G23" s="4" t="inlineStr"/>
       <c r="H23" s="3" t="inlineStr"/>
-      <c r="I23" s="3" t="inlineStr"/>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>Evaluation Engine</t>
+        </is>
+      </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
           <t>§4.2 SD-03; §4.3 API-15</t>
@@ -1571,7 +1659,11 @@
       </c>
       <c r="G24" s="2" t="inlineStr"/>
       <c r="H24" s="3" t="inlineStr"/>
-      <c r="I24" s="3" t="inlineStr"/>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>Result &amp; Analytics Service</t>
+        </is>
+      </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
           <t>§4.3 API-16; §4.5 Result page</t>
@@ -1616,7 +1708,11 @@
       </c>
       <c r="G25" s="4" t="inlineStr"/>
       <c r="H25" s="3" t="inlineStr"/>
-      <c r="I25" s="3" t="inlineStr"/>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Result &amp; Analytics Service</t>
+        </is>
+      </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
           <t>§4.3 API-17</t>
@@ -1661,7 +1757,11 @@
       </c>
       <c r="G26" s="2" t="inlineStr"/>
       <c r="H26" s="3" t="inlineStr"/>
-      <c r="I26" s="3" t="inlineStr"/>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>Result &amp; Analytics Service</t>
+        </is>
+      </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
           <t>§4.3 API-18</t>
@@ -1706,7 +1806,11 @@
       </c>
       <c r="G27" s="4" t="inlineStr"/>
       <c r="H27" s="3" t="inlineStr"/>
-      <c r="I27" s="3" t="inlineStr"/>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>Notification Service</t>
+        </is>
+      </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
           <t>§4.2 SD-03; §4.3 API-10, API-19</t>
@@ -1751,7 +1855,11 @@
       </c>
       <c r="G28" s="2" t="inlineStr"/>
       <c r="H28" s="3" t="inlineStr"/>
-      <c r="I28" s="3" t="inlineStr"/>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>Audit &amp; Logging Service</t>
+        </is>
+      </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
           <t>§4.3 API-20; §4.4.2 Audit log</t>
@@ -1792,7 +1900,11 @@
       <c r="F29" s="4" t="inlineStr"/>
       <c r="G29" s="4" t="inlineStr"/>
       <c r="H29" s="3" t="inlineStr"/>
-      <c r="I29" s="3" t="inlineStr"/>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>All layers (esp. API + MongoDB)</t>
+        </is>
+      </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
           <t>§4.4.3 M-01</t>
@@ -1833,7 +1945,11 @@
       <c r="F30" s="2" t="inlineStr"/>
       <c r="G30" s="2" t="inlineStr"/>
       <c r="H30" s="3" t="inlineStr"/>
-      <c r="I30" s="3" t="inlineStr"/>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>Exam Management Service + Data Access</t>
+        </is>
+      </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
           <t>§4.3 API-13; §4.4.3 M-02</t>
@@ -1874,7 +1990,11 @@
       <c r="F31" s="4" t="inlineStr"/>
       <c r="G31" s="4" t="inlineStr"/>
       <c r="H31" s="3" t="inlineStr"/>
-      <c r="I31" s="3" t="inlineStr"/>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>Evaluation Engine</t>
+        </is>
+      </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
           <t>§4.2 SD-03; §4.4.3 M-03</t>
@@ -1915,7 +2035,11 @@
       <c r="F32" s="2" t="inlineStr"/>
       <c r="G32" s="2" t="inlineStr"/>
       <c r="H32" s="3" t="inlineStr"/>
-      <c r="I32" s="3" t="inlineStr"/>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>Deployment + Monitoring</t>
+        </is>
+      </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
           <t>§4.3 API-21; §4.4.3 M-04, M-05</t>
@@ -1956,7 +2080,11 @@
       <c r="F33" s="4" t="inlineStr"/>
       <c r="G33" s="4" t="inlineStr"/>
       <c r="H33" s="3" t="inlineStr"/>
-      <c r="I33" s="3" t="inlineStr"/>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>Exam Management Service</t>
+        </is>
+      </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
           <t>§4.2 SD-02, SD-03; §4.4.1 exam-page resilience</t>
@@ -1997,7 +2125,11 @@
       <c r="F34" s="2" t="inlineStr"/>
       <c r="G34" s="2" t="inlineStr"/>
       <c r="H34" s="3" t="inlineStr"/>
-      <c r="I34" s="3" t="inlineStr"/>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>TBD (P3) – not in SAD 3.8</t>
+        </is>
+      </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
           <t>§4.1 jobs/backup; §4.4.3 M-08</t>
@@ -2038,7 +2170,11 @@
       <c r="F35" s="4" t="inlineStr"/>
       <c r="G35" s="4" t="inlineStr"/>
       <c r="H35" s="3" t="inlineStr"/>
-      <c r="I35" s="3" t="inlineStr"/>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>TBD (P3) – not in SAD 3.8</t>
+        </is>
+      </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
           <t>§4.5 Student dashboard (3 clicks)</t>
@@ -2079,7 +2215,11 @@
       <c r="F36" s="2" t="inlineStr"/>
       <c r="G36" s="2" t="inlineStr"/>
       <c r="H36" s="3" t="inlineStr"/>
-      <c r="I36" s="3" t="inlineStr"/>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>TBD (P3) – not in SAD 3.8</t>
+        </is>
+      </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
           <t>§4.5 Accessibility</t>
@@ -2120,7 +2260,11 @@
       <c r="F37" s="4" t="inlineStr"/>
       <c r="G37" s="4" t="inlineStr"/>
       <c r="H37" s="3" t="inlineStr"/>
-      <c r="I37" s="3" t="inlineStr"/>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>TBD (P3) – not in SAD 3.8</t>
+        </is>
+      </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
           <t>§4.5 Accessibility &amp; compatibility</t>
@@ -2161,7 +2305,11 @@
       <c r="F38" s="2" t="inlineStr"/>
       <c r="G38" s="2" t="inlineStr"/>
       <c r="H38" s="3" t="inlineStr"/>
-      <c r="I38" s="3" t="inlineStr"/>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>Exam Management Service</t>
+        </is>
+      </c>
       <c r="J38" s="3" t="inlineStr">
         <is>
           <t>§4.2 SD-02 (server time offset); §4.3 API-12</t>
@@ -2202,7 +2350,11 @@
       <c r="F39" s="4" t="inlineStr"/>
       <c r="G39" s="4" t="inlineStr"/>
       <c r="H39" s="3" t="inlineStr"/>
-      <c r="I39" s="3" t="inlineStr"/>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>TBD (P3) – not in SAD 3.8</t>
+        </is>
+      </c>
       <c r="J39" s="3" t="inlineStr">
         <is>
           <t>§4.1 data entities &amp; indexes</t>
@@ -2243,7 +2395,11 @@
       <c r="F40" s="2" t="inlineStr"/>
       <c r="G40" s="2" t="inlineStr"/>
       <c r="H40" s="3" t="inlineStr"/>
-      <c r="I40" s="3" t="inlineStr"/>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>TBD (P3) – not in SAD 3.8</t>
+        </is>
+      </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
           <t>§4.1 module structure</t>
@@ -2284,7 +2440,11 @@
       <c r="F41" s="4" t="inlineStr"/>
       <c r="G41" s="4" t="inlineStr"/>
       <c r="H41" s="3" t="inlineStr"/>
-      <c r="I41" s="3" t="inlineStr"/>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>TBD (P3) – not in SAD 3.8</t>
+        </is>
+      </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
           <t>§4.7 item 5 (Docker Compose)</t>
@@ -2325,7 +2485,11 @@
       <c r="F42" s="2" t="inlineStr"/>
       <c r="G42" s="2" t="inlineStr"/>
       <c r="H42" s="3" t="inlineStr"/>
-      <c r="I42" s="3" t="inlineStr"/>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>TBD (P3) – not in SAD 3.8</t>
+        </is>
+      </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
           <t>§4.3 API-07; §4.1 data entities</t>
@@ -2370,7 +2534,11 @@
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr"/>
-      <c r="I43" s="3" t="inlineStr"/>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>Authentication &amp; Authorization Service</t>
+        </is>
+      </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
           <t>§4.2 SD-01; §4.3 API-03</t>
@@ -2415,7 +2583,11 @@
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr"/>
-      <c r="I44" s="3" t="inlineStr"/>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>Authentication &amp; Authorization Service</t>
+        </is>
+      </c>
       <c r="J44" s="3" t="inlineStr">
         <is>
           <t>§4.3 API-01, API-06</t>
@@ -2460,7 +2632,11 @@
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr"/>
-      <c r="I45" s="3" t="inlineStr"/>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>Authentication &amp; Authorization Service</t>
+        </is>
+      </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
           <t>§4.2 SD-01; §4.3 API-03 (423)</t>
@@ -2505,7 +2681,11 @@
         </is>
       </c>
       <c r="H46" s="3" t="inlineStr"/>
-      <c r="I46" s="3" t="inlineStr"/>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>Authentication &amp; Authorization Service</t>
+        </is>
+      </c>
       <c r="J46" s="3" t="inlineStr">
         <is>
           <t>§4.2 SD-01, SD-02; §4.3.1 conventions</t>
@@ -2550,7 +2730,11 @@
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr"/>
-      <c r="I47" s="3" t="inlineStr"/>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>API Layer + Infrastructure</t>
+        </is>
+      </c>
       <c r="J47" s="3" t="inlineStr">
         <is>
           <t>§4.3.1 conventions</t>
@@ -2595,7 +2779,11 @@
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr"/>
-      <c r="I48" s="3" t="inlineStr"/>
+      <c r="I48" s="3" t="inlineStr">
+        <is>
+          <t>Authentication &amp; Authorization Service</t>
+        </is>
+      </c>
       <c r="J48" s="3" t="inlineStr">
         <is>
           <t>§4.2 SD-01; §4.3 API-03</t>
@@ -2640,7 +2828,11 @@
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr"/>
-      <c r="I49" s="3" t="inlineStr"/>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>Exam Management + Evaluation Engine</t>
+        </is>
+      </c>
       <c r="J49" s="3" t="inlineStr">
         <is>
           <t>§4.2 SD-02; §4.3 API-12, API-16</t>
@@ -2685,7 +2877,11 @@
         </is>
       </c>
       <c r="H50" s="3" t="inlineStr"/>
-      <c r="I50" s="3" t="inlineStr"/>
+      <c r="I50" s="3" t="inlineStr">
+        <is>
+          <t>API Layer + All Services</t>
+        </is>
+      </c>
       <c r="J50" s="3" t="inlineStr">
         <is>
           <t>§4.3.1 conventions; §4.4.1</t>
@@ -2730,7 +2926,11 @@
         </is>
       </c>
       <c r="H51" s="3" t="inlineStr"/>
-      <c r="I51" s="3" t="inlineStr"/>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>Exam Management Service</t>
+        </is>
+      </c>
       <c r="J51" s="3" t="inlineStr">
         <is>
           <t>§4.2 SD-02, SD-03; §4.3 API-13, API-15</t>
@@ -2775,7 +2975,11 @@
         </is>
       </c>
       <c r="H52" s="3" t="inlineStr"/>
-      <c r="I52" s="3" t="inlineStr"/>
+      <c r="I52" s="3" t="inlineStr">
+        <is>
+          <t>API Layer</t>
+        </is>
+      </c>
       <c r="J52" s="3" t="inlineStr">
         <is>
           <t>§4.2 SD-01; §4.3 API-03, API-05 (429)</t>
@@ -2820,7 +3024,11 @@
         </is>
       </c>
       <c r="H53" s="3" t="inlineStr"/>
-      <c r="I53" s="3" t="inlineStr"/>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>Audit &amp; Logging Service</t>
+        </is>
+      </c>
       <c r="J53" s="3" t="inlineStr">
         <is>
           <t>§4.4.2 Logging; §4.3 API-20</t>
@@ -2865,7 +3073,11 @@
         </is>
       </c>
       <c r="H54" s="3" t="inlineStr"/>
-      <c r="I54" s="3" t="inlineStr"/>
+      <c r="I54" s="3" t="inlineStr">
+        <is>
+          <t>Data Access Layer + MongoDB</t>
+        </is>
+      </c>
       <c r="J54" s="3" t="inlineStr">
         <is>
           <t>§4.1 data entities (encrypted fields)</t>

</xml_diff>

<commit_message>
SRS v1.2 final: replace old files with final versions
</commit_message>
<xml_diff>
--- a/SRS/RTM_Online_Exam_Portal.xlsx
+++ b/SRS/RTM_Online_Exam_Portal.xlsx
@@ -580,7 +580,11 @@
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="3" t="inlineStr"/>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-001</t>
+        </is>
+      </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
           <t>Authentication &amp; Authorization Service</t>
@@ -629,7 +633,11 @@
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr"/>
-      <c r="H3" s="3" t="inlineStr"/>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-001</t>
+        </is>
+      </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Authentication &amp; Authorization Service + Notification Service</t>
@@ -678,7 +686,11 @@
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="3" t="inlineStr"/>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-001</t>
+        </is>
+      </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Authentication &amp; Authorization Service</t>
@@ -727,7 +739,11 @@
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr"/>
-      <c r="H5" s="3" t="inlineStr"/>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-001</t>
+        </is>
+      </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Authentication &amp; Authorization Service</t>
@@ -776,7 +792,11 @@
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="3" t="inlineStr"/>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-002</t>
+        </is>
+      </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
           <t>Authentication &amp; Authorization Service + Notification Service</t>
@@ -825,7 +845,11 @@
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr"/>
-      <c r="H7" s="3" t="inlineStr"/>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-003</t>
+        </is>
+      </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
           <t>Authentication &amp; Authorization Service</t>
@@ -874,7 +898,11 @@
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="3" t="inlineStr"/>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-004</t>
+        </is>
+      </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
           <t>Question Bank Service</t>
@@ -923,7 +951,11 @@
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr"/>
-      <c r="H9" s="3" t="inlineStr"/>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-004</t>
+        </is>
+      </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
           <t>Exam Management Service</t>
@@ -972,7 +1004,11 @@
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="3" t="inlineStr"/>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-004</t>
+        </is>
+      </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
           <t>Exam Management Service</t>
@@ -1021,7 +1057,11 @@
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr"/>
-      <c r="H11" s="3" t="inlineStr"/>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-004</t>
+        </is>
+      </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
           <t>Exam Management Service + Evaluation Engine</t>
@@ -1070,7 +1110,11 @@
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="3" t="inlineStr"/>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-005</t>
+        </is>
+      </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
           <t>Exam Management Service + Notification Service</t>
@@ -1119,7 +1163,11 @@
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr"/>
-      <c r="H13" s="3" t="inlineStr"/>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-004</t>
+        </is>
+      </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
           <t>Exam Management Service</t>
@@ -1168,7 +1216,11 @@
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
-      <c r="H14" s="3" t="inlineStr"/>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-005</t>
+        </is>
+      </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
           <t>Exam Management Service</t>
@@ -1217,7 +1269,11 @@
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr"/>
-      <c r="H15" s="3" t="inlineStr"/>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-006</t>
+        </is>
+      </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
           <t>Exam Management Service</t>
@@ -1266,7 +1322,11 @@
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr"/>
-      <c r="H16" s="3" t="inlineStr"/>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-006</t>
+        </is>
+      </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
           <t>Exam Management Service + Presentation Layer</t>
@@ -1315,7 +1375,11 @@
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr"/>
-      <c r="H17" s="3" t="inlineStr"/>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-006</t>
+        </is>
+      </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
           <t>Exam Management Service</t>
@@ -1364,7 +1428,11 @@
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr"/>
-      <c r="H18" s="3" t="inlineStr"/>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-007</t>
+        </is>
+      </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
           <t>Exam Management Service</t>
@@ -1413,7 +1481,11 @@
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr"/>
-      <c r="H19" s="3" t="inlineStr"/>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-007</t>
+        </is>
+      </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
           <t>Exam Management Service</t>
@@ -1462,7 +1534,11 @@
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="3" t="inlineStr"/>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-006, TC-OE-008</t>
+        </is>
+      </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
           <t>Exam Management Service</t>
@@ -1511,7 +1587,11 @@
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr"/>
-      <c r="H21" s="3" t="inlineStr"/>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-006, TC-OE-008</t>
+        </is>
+      </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
           <t>Exam Management Service</t>
@@ -1560,7 +1640,11 @@
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr"/>
-      <c r="H22" s="3" t="inlineStr"/>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-006</t>
+        </is>
+      </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
           <t>Exam Management Service + Audit &amp; Logging Service</t>
@@ -1609,7 +1693,11 @@
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr"/>
-      <c r="H23" s="3" t="inlineStr"/>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-008</t>
+        </is>
+      </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
           <t>Evaluation Engine</t>
@@ -1658,7 +1746,11 @@
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
-      <c r="H24" s="3" t="inlineStr"/>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-009</t>
+        </is>
+      </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
           <t>Result &amp; Analytics Service</t>
@@ -1707,7 +1799,11 @@
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr"/>
-      <c r="H25" s="3" t="inlineStr"/>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-009</t>
+        </is>
+      </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
           <t>Result &amp; Analytics Service</t>
@@ -1756,7 +1852,11 @@
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr"/>
-      <c r="H26" s="3" t="inlineStr"/>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-009</t>
+        </is>
+      </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
           <t>Result &amp; Analytics Service</t>
@@ -1805,7 +1905,11 @@
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr"/>
-      <c r="H27" s="3" t="inlineStr"/>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-005</t>
+        </is>
+      </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
           <t>Notification Service</t>
@@ -1854,7 +1958,11 @@
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr"/>
-      <c r="H28" s="3" t="inlineStr"/>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-003, TC-OE-009</t>
+        </is>
+      </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
           <t>Audit &amp; Logging Service</t>
@@ -1899,7 +2007,11 @@
       </c>
       <c r="F29" s="4" t="inlineStr"/>
       <c r="G29" s="4" t="inlineStr"/>
-      <c r="H29" s="3" t="inlineStr"/>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-010</t>
+        </is>
+      </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
           <t>All layers (esp. API + MongoDB)</t>
@@ -1944,7 +2056,11 @@
       </c>
       <c r="F30" s="2" t="inlineStr"/>
       <c r="G30" s="2" t="inlineStr"/>
-      <c r="H30" s="3" t="inlineStr"/>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-007, TC-OE-010</t>
+        </is>
+      </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
           <t>Exam Management Service + Data Access</t>
@@ -1989,7 +2105,11 @@
       </c>
       <c r="F31" s="4" t="inlineStr"/>
       <c r="G31" s="4" t="inlineStr"/>
-      <c r="H31" s="3" t="inlineStr"/>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-008, TC-OE-010</t>
+        </is>
+      </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
           <t>Evaluation Engine</t>
@@ -2034,7 +2154,11 @@
       </c>
       <c r="F32" s="2" t="inlineStr"/>
       <c r="G32" s="2" t="inlineStr"/>
-      <c r="H32" s="3" t="inlineStr"/>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-010</t>
+        </is>
+      </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
           <t>Deployment + Monitoring</t>
@@ -2079,7 +2203,11 @@
       </c>
       <c r="F33" s="4" t="inlineStr"/>
       <c r="G33" s="4" t="inlineStr"/>
-      <c r="H33" s="3" t="inlineStr"/>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-007</t>
+        </is>
+      </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
           <t>Exam Management Service</t>
@@ -2124,10 +2252,14 @@
       </c>
       <c r="F34" s="2" t="inlineStr"/>
       <c r="G34" s="2" t="inlineStr"/>
-      <c r="H34" s="3" t="inlineStr"/>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-009</t>
+        </is>
+      </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>TBD (P3) – not in SAD 3.8</t>
+          <t>MongoDB + Deployment (daily backup job)</t>
         </is>
       </c>
       <c r="J34" s="3" t="inlineStr">
@@ -2169,10 +2301,14 @@
       </c>
       <c r="F35" s="4" t="inlineStr"/>
       <c r="G35" s="4" t="inlineStr"/>
-      <c r="H35" s="3" t="inlineStr"/>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-005</t>
+        </is>
+      </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>TBD (P3) – not in SAD 3.8</t>
+          <t>Presentation Layer (React)</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
@@ -2214,10 +2350,14 @@
       </c>
       <c r="F36" s="2" t="inlineStr"/>
       <c r="G36" s="2" t="inlineStr"/>
-      <c r="H36" s="3" t="inlineStr"/>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-006</t>
+        </is>
+      </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>TBD (P3) – not in SAD 3.8</t>
+          <t>Presentation Layer (React)</t>
         </is>
       </c>
       <c r="J36" s="3" t="inlineStr">
@@ -2259,10 +2399,14 @@
       </c>
       <c r="F37" s="4" t="inlineStr"/>
       <c r="G37" s="4" t="inlineStr"/>
-      <c r="H37" s="3" t="inlineStr"/>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-006</t>
+        </is>
+      </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>TBD (P3) – not in SAD 3.8</t>
+          <t>Presentation Layer (React)</t>
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr">
@@ -2304,7 +2448,11 @@
       </c>
       <c r="F38" s="2" t="inlineStr"/>
       <c r="G38" s="2" t="inlineStr"/>
-      <c r="H38" s="3" t="inlineStr"/>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-006</t>
+        </is>
+      </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
           <t>Exam Management Service</t>
@@ -2349,10 +2497,14 @@
       </c>
       <c r="F39" s="4" t="inlineStr"/>
       <c r="G39" s="4" t="inlineStr"/>
-      <c r="H39" s="3" t="inlineStr"/>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-010</t>
+        </is>
+      </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>TBD (P3) – not in SAD 3.8</t>
+          <t>Data Access Layer + MongoDB (indexes)</t>
         </is>
       </c>
       <c r="J39" s="3" t="inlineStr">
@@ -2394,10 +2546,14 @@
       </c>
       <c r="F40" s="2" t="inlineStr"/>
       <c r="G40" s="2" t="inlineStr"/>
-      <c r="H40" s="3" t="inlineStr"/>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-009, TC-OE-010</t>
+        </is>
+      </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>TBD (P3) – not in SAD 3.8</t>
+          <t>All Business Services (modular layered structure)</t>
         </is>
       </c>
       <c r="J40" s="3" t="inlineStr">
@@ -2439,10 +2595,14 @@
       </c>
       <c r="F41" s="4" t="inlineStr"/>
       <c r="G41" s="4" t="inlineStr"/>
-      <c r="H41" s="3" t="inlineStr"/>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-010</t>
+        </is>
+      </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>TBD (P3) – not in SAD 3.8</t>
+          <t>Deployment (Docker Compose: React, Node.js, MongoDB)</t>
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr">
@@ -2484,10 +2644,14 @@
       </c>
       <c r="F42" s="2" t="inlineStr"/>
       <c r="G42" s="2" t="inlineStr"/>
-      <c r="H42" s="3" t="inlineStr"/>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-009</t>
+        </is>
+      </c>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>TBD (P3) – not in SAD 3.8</t>
+          <t>Authentication &amp; Authorization Service + Data Access Layer + MongoDB</t>
         </is>
       </c>
       <c r="J42" s="3" t="inlineStr">
@@ -2533,7 +2697,11 @@
           <t>SO-OE-003</t>
         </is>
       </c>
-      <c r="H43" s="3" t="inlineStr"/>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-001</t>
+        </is>
+      </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
           <t>Authentication &amp; Authorization Service</t>
@@ -2582,7 +2750,11 @@
           <t>SO-OE-003</t>
         </is>
       </c>
-      <c r="H44" s="3" t="inlineStr"/>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-001</t>
+        </is>
+      </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
           <t>Authentication &amp; Authorization Service</t>
@@ -2631,7 +2803,11 @@
           <t>SO-OE-003</t>
         </is>
       </c>
-      <c r="H45" s="3" t="inlineStr"/>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-002</t>
+        </is>
+      </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
           <t>Authentication &amp; Authorization Service</t>
@@ -2680,7 +2856,11 @@
           <t>SO-OE-003</t>
         </is>
       </c>
-      <c r="H46" s="3" t="inlineStr"/>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-003</t>
+        </is>
+      </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
           <t>Authentication &amp; Authorization Service</t>
@@ -2729,7 +2909,11 @@
           <t>SO-OE-001</t>
         </is>
       </c>
-      <c r="H47" s="3" t="inlineStr"/>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-001</t>
+        </is>
+      </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
           <t>API Layer + Infrastructure</t>
@@ -2778,7 +2962,11 @@
           <t>SO-OE-003</t>
         </is>
       </c>
-      <c r="H48" s="3" t="inlineStr"/>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-001</t>
+        </is>
+      </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
           <t>Authentication &amp; Authorization Service</t>
@@ -2827,7 +3015,11 @@
           <t>SO-OE-001</t>
         </is>
       </c>
-      <c r="H49" s="3" t="inlineStr"/>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-006</t>
+        </is>
+      </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
           <t>Exam Management + Evaluation Engine</t>
@@ -2876,7 +3068,11 @@
           <t>SO-OE-002</t>
         </is>
       </c>
-      <c r="H50" s="3" t="inlineStr"/>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-004</t>
+        </is>
+      </c>
       <c r="I50" s="3" t="inlineStr">
         <is>
           <t>API Layer + All Services</t>
@@ -2925,7 +3121,11 @@
           <t>SO-OE-002</t>
         </is>
       </c>
-      <c r="H51" s="3" t="inlineStr"/>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-006</t>
+        </is>
+      </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
           <t>Exam Management Service</t>
@@ -2974,7 +3174,11 @@
           <t>SO-OE-004</t>
         </is>
       </c>
-      <c r="H52" s="3" t="inlineStr"/>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-002</t>
+        </is>
+      </c>
       <c r="I52" s="3" t="inlineStr">
         <is>
           <t>API Layer</t>
@@ -3023,7 +3227,11 @@
           <t>SO-OE-005</t>
         </is>
       </c>
-      <c r="H53" s="3" t="inlineStr"/>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-003, TC-OE-005, TC-OE-009</t>
+        </is>
+      </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
           <t>Audit &amp; Logging Service</t>
@@ -3072,7 +3280,11 @@
           <t>SO-OE-001</t>
         </is>
       </c>
-      <c r="H54" s="3" t="inlineStr"/>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>TC-OE-009</t>
+        </is>
+      </c>
       <c r="I54" s="3" t="inlineStr">
         <is>
           <t>Data Access Layer + MongoDB</t>

</xml_diff>